<commit_message>
#15 BOM review Complete
</commit_message>
<xml_diff>
--- a/BOM/Client-BOM.xlsx
+++ b/BOM/Client-BOM.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="436" uniqueCount="288">
   <si>
     <t>Description</t>
   </si>
@@ -880,15 +880,9 @@
     <t>Aliexpress</t>
   </si>
   <si>
-    <t>40 Pin Breakable Header 100 pieces per lot</t>
-  </si>
-  <si>
     <t>Verical</t>
   </si>
   <si>
-    <t>MOQ Issue</t>
-  </si>
-  <si>
     <t>UTSource</t>
   </si>
   <si>
@@ -920,6 +914,12 @@
   </si>
   <si>
     <t xml:space="preserve">PANASONIC </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rochester </t>
+  </si>
+  <si>
+    <t>Arrow</t>
   </si>
 </sst>
 </file>
@@ -1465,7 +1465,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1716,9 +1716,6 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="22" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1804,35 +1801,35 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2143,29 +2140,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="123" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="117"/>
-      <c r="L1" s="117"/>
-      <c r="M1" s="117"/>
-      <c r="N1" s="117"/>
-      <c r="O1" s="117"/>
-      <c r="P1" s="117"/>
-      <c r="Q1" s="117"/>
-      <c r="R1" s="117"/>
-      <c r="S1" s="117"/>
-      <c r="T1" s="117"/>
-      <c r="U1" s="118"/>
+      <c r="B1" s="124"/>
+      <c r="C1" s="124"/>
+      <c r="D1" s="124"/>
+      <c r="E1" s="124"/>
+      <c r="F1" s="124"/>
+      <c r="G1" s="124"/>
+      <c r="H1" s="124"/>
+      <c r="I1" s="124"/>
+      <c r="J1" s="124"/>
+      <c r="K1" s="124"/>
+      <c r="L1" s="124"/>
+      <c r="M1" s="124"/>
+      <c r="N1" s="124"/>
+      <c r="O1" s="124"/>
+      <c r="P1" s="124"/>
+      <c r="Q1" s="124"/>
+      <c r="R1" s="124"/>
+      <c r="S1" s="124"/>
+      <c r="T1" s="124"/>
+      <c r="U1" s="125"/>
     </row>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -2236,7 +2233,7 @@
       <c r="A3" s="16">
         <v>1</v>
       </c>
-      <c r="B3" s="119" t="s">
+      <c r="B3" s="118" t="s">
         <v>14</v>
       </c>
       <c r="C3" s="23" t="s">
@@ -2248,7 +2245,7 @@
       <c r="E3" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="F3" s="109" t="s">
+      <c r="F3" s="108" t="s">
         <v>85</v>
       </c>
       <c r="G3" s="1" t="s">
@@ -2304,7 +2301,7 @@
       <c r="A4" s="16">
         <v>2</v>
       </c>
-      <c r="B4" s="120"/>
+      <c r="B4" s="119"/>
       <c r="C4" s="28" t="s">
         <v>86</v>
       </c>
@@ -2355,10 +2352,12 @@
         <f t="shared" ref="R4:R52" si="1">Q4*L4</f>
         <v>33</v>
       </c>
-      <c r="S4" s="35"/>
+      <c r="S4" s="35">
+        <v>3.1475409836065601E-2</v>
+      </c>
       <c r="T4" s="35">
         <f t="shared" ref="T4:T52" si="2">S4*M4</f>
-        <v>0</v>
+        <v>192.00000000000017</v>
       </c>
       <c r="U4" s="36"/>
       <c r="V4" s="3"/>
@@ -2368,7 +2367,7 @@
       <c r="A5" s="16">
         <v>3</v>
       </c>
-      <c r="B5" s="120"/>
+      <c r="B5" s="119"/>
       <c r="C5" s="28" t="s">
         <v>90</v>
       </c>
@@ -2397,7 +2396,7 @@
         <v>20</v>
       </c>
       <c r="L5" s="33">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="M5" s="33">
         <v>3100</v>
@@ -2417,14 +2416,14 @@
       </c>
       <c r="R5" s="35">
         <f t="shared" si="1"/>
-        <v>20.097000000000001</v>
+        <v>19.488</v>
       </c>
       <c r="S5" s="38">
-        <v>4.7600000000000003E-2</v>
+        <v>5.5899999999999998E-2</v>
       </c>
       <c r="T5" s="35">
         <f t="shared" si="2"/>
-        <v>147.56</v>
+        <v>173.29</v>
       </c>
       <c r="U5" s="25"/>
       <c r="V5" s="3"/>
@@ -2434,7 +2433,7 @@
       <c r="A6" s="16">
         <v>4</v>
       </c>
-      <c r="B6" s="120"/>
+      <c r="B6" s="119"/>
       <c r="C6" s="28" t="s">
         <v>93</v>
       </c>
@@ -2460,7 +2459,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="33">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="L6" s="33">
         <v>150</v>
@@ -2476,7 +2475,7 @@
       </c>
       <c r="P6" s="35">
         <f t="shared" si="0"/>
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="Q6" s="35">
         <v>4.0000000000000001E-3</v>
@@ -2500,7 +2499,7 @@
       <c r="A7" s="16">
         <v>5</v>
       </c>
-      <c r="B7" s="120"/>
+      <c r="B7" s="119"/>
       <c r="C7" s="28" t="s">
         <v>95</v>
       </c>
@@ -2526,7 +2525,7 @@
         <v>2</v>
       </c>
       <c r="K7" s="33">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="L7" s="33">
         <v>250</v>
@@ -2542,7 +2541,7 @@
       </c>
       <c r="P7" s="35">
         <f t="shared" si="0"/>
-        <v>0.97</v>
+        <v>0.48499999999999999</v>
       </c>
       <c r="Q7" s="35">
         <v>9.7000000000000003E-3</v>
@@ -2566,7 +2565,7 @@
       <c r="A8" s="16">
         <v>6</v>
       </c>
-      <c r="B8" s="120"/>
+      <c r="B8" s="119"/>
       <c r="C8" s="28" t="s">
         <v>98</v>
       </c>
@@ -2632,7 +2631,7 @@
       <c r="A9" s="16">
         <v>7</v>
       </c>
-      <c r="B9" s="120"/>
+      <c r="B9" s="119"/>
       <c r="C9" s="28" t="s">
         <v>102</v>
       </c>
@@ -2670,25 +2669,25 @@
         <v>250</v>
       </c>
       <c r="O9" s="35">
-        <v>8.8499999999999995E-2</v>
+        <v>9.06E-2</v>
       </c>
       <c r="P9" s="35">
         <f t="shared" si="0"/>
-        <v>1.3274999999999999</v>
+        <v>1.359</v>
       </c>
       <c r="Q9" s="35">
-        <v>6.5699999999999995E-2</v>
+        <v>6.83E-2</v>
       </c>
       <c r="R9" s="35">
         <f t="shared" si="1"/>
-        <v>15.110999999999999</v>
+        <v>15.709</v>
       </c>
       <c r="S9" s="35">
-        <v>6.2199999999999998E-2</v>
+        <v>6.4799999999999996E-2</v>
       </c>
       <c r="T9" s="35">
         <f t="shared" si="2"/>
-        <v>130.62</v>
+        <v>136.07999999999998</v>
       </c>
       <c r="U9" s="25"/>
       <c r="V9" s="3"/>
@@ -2698,7 +2697,7 @@
       <c r="A10" s="16">
         <v>8</v>
       </c>
-      <c r="B10" s="121"/>
+      <c r="B10" s="120"/>
       <c r="C10" s="39" t="s">
         <v>105</v>
       </c>
@@ -2708,7 +2707,7 @@
       <c r="E10" s="40" t="s">
         <v>84</v>
       </c>
-      <c r="F10" s="108" t="s">
+      <c r="F10" s="107" t="s">
         <v>107</v>
       </c>
       <c r="G10" s="41" t="s">
@@ -2764,10 +2763,10 @@
       <c r="A11" s="16">
         <v>9</v>
       </c>
-      <c r="B11" s="119" t="s">
+      <c r="B11" s="118" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="107" t="s">
+      <c r="C11" s="106" t="s">
         <v>252</v>
       </c>
       <c r="D11" s="63" t="s">
@@ -2792,16 +2791,13 @@
         <v>1</v>
       </c>
       <c r="K11" s="66">
-        <f t="shared" ref="K11:K50" si="3">J11*5</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L11" s="66">
-        <f t="shared" ref="L11:L51" si="4">J11*100</f>
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="M11" s="66">
-        <f t="shared" ref="M11:M50" si="5">J11*1000</f>
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="N11" s="67" t="s">
         <v>250</v>
@@ -2811,21 +2807,21 @@
       </c>
       <c r="P11" s="68">
         <f t="shared" si="0"/>
-        <v>0.3775</v>
+        <v>0.755</v>
       </c>
       <c r="Q11" s="68">
         <v>5.79E-2</v>
       </c>
       <c r="R11" s="68">
         <f t="shared" si="1"/>
-        <v>5.79</v>
+        <v>6.9480000000000004</v>
       </c>
       <c r="S11" s="68">
-        <v>4.53E-2</v>
+        <v>4.2200000000000001E-2</v>
       </c>
       <c r="T11" s="68">
         <f t="shared" si="2"/>
-        <v>45.3</v>
+        <v>46.42</v>
       </c>
       <c r="U11" s="83"/>
       <c r="V11" s="3"/>
@@ -2835,7 +2831,7 @@
       <c r="A12" s="16">
         <v>10</v>
       </c>
-      <c r="B12" s="120"/>
+      <c r="B12" s="119"/>
       <c r="C12" s="28" t="s">
         <v>110</v>
       </c>
@@ -2864,12 +2860,10 @@
         <v>20</v>
       </c>
       <c r="L12" s="33">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="M12" s="33">
-        <f t="shared" si="5"/>
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="N12" s="34" t="s">
         <v>250</v>
@@ -2886,14 +2880,14 @@
       </c>
       <c r="R12" s="35">
         <f t="shared" si="1"/>
-        <v>1.83</v>
+        <v>2.1960000000000002</v>
       </c>
       <c r="S12" s="35">
         <v>1.23E-2</v>
       </c>
       <c r="T12" s="35">
         <f t="shared" si="2"/>
-        <v>12.3</v>
+        <v>13.53</v>
       </c>
       <c r="U12" s="36"/>
       <c r="V12" s="3"/>
@@ -2903,7 +2897,7 @@
       <c r="A13" s="16">
         <v>11</v>
       </c>
-      <c r="B13" s="121"/>
+      <c r="B13" s="120"/>
       <c r="C13" s="39" t="s">
         <v>113</v>
       </c>
@@ -2929,16 +2923,13 @@
         <v>2</v>
       </c>
       <c r="K13" s="44">
-        <f t="shared" si="3"/>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="L13" s="44">
-        <f t="shared" si="4"/>
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="M13" s="44">
-        <f t="shared" si="5"/>
-        <v>2000</v>
+        <v>2100</v>
       </c>
       <c r="N13" s="45" t="s">
         <v>250</v>
@@ -2948,21 +2939,21 @@
       </c>
       <c r="P13" s="46">
         <f t="shared" si="0"/>
-        <v>1.087</v>
+        <v>1.6305000000000001</v>
       </c>
       <c r="Q13" s="46">
         <v>7.7200000000000005E-2</v>
       </c>
       <c r="R13" s="46">
         <f t="shared" si="1"/>
-        <v>15.440000000000001</v>
+        <v>17.756</v>
       </c>
       <c r="S13" s="46">
         <v>7.2300000000000003E-2</v>
       </c>
       <c r="T13" s="46">
         <f t="shared" si="2"/>
-        <v>144.6</v>
+        <v>151.83000000000001</v>
       </c>
       <c r="U13" s="26"/>
       <c r="V13" s="3"/>
@@ -2972,7 +2963,7 @@
       <c r="A14" s="16">
         <v>12</v>
       </c>
-      <c r="B14" s="119" t="s">
+      <c r="B14" s="118" t="s">
         <v>30</v>
       </c>
       <c r="C14" s="62" t="s">
@@ -3003,36 +2994,34 @@
         <v>10</v>
       </c>
       <c r="L14" s="66">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="M14" s="66">
-        <f t="shared" si="5"/>
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="N14" s="67" t="s">
         <v>250</v>
       </c>
       <c r="O14" s="68">
-        <v>4.9000000000000002E-2</v>
+        <v>4.5900000000000003E-2</v>
       </c>
       <c r="P14" s="68">
         <f t="shared" si="0"/>
-        <v>0.49</v>
+        <v>0.45900000000000002</v>
       </c>
       <c r="Q14" s="68">
-        <v>3.9100000000000003E-2</v>
+        <v>3.5999999999999997E-2</v>
       </c>
       <c r="R14" s="68">
         <f t="shared" si="1"/>
-        <v>3.91</v>
+        <v>4.3199999999999994</v>
       </c>
       <c r="S14" s="68">
-        <v>2.4899999999999999E-2</v>
+        <v>3.2399999999999998E-2</v>
       </c>
       <c r="T14" s="68">
         <f t="shared" si="2"/>
-        <v>24.9</v>
+        <v>35.64</v>
       </c>
       <c r="U14" s="69"/>
       <c r="V14" s="3"/>
@@ -3042,7 +3031,7 @@
       <c r="A15" s="16">
         <v>13</v>
       </c>
-      <c r="B15" s="120"/>
+      <c r="B15" s="119"/>
       <c r="C15" s="70" t="s">
         <v>222</v>
       </c>
@@ -3064,42 +3053,43 @@
       <c r="I15" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="J15" s="111">
+      <c r="J15" s="110">
         <v>1</v>
       </c>
       <c r="K15" s="33">
-        <v>60</v>
+        <v>113</v>
       </c>
       <c r="L15" s="33">
-        <v>120</v>
-      </c>
-      <c r="M15" s="112">
+        <v>113</v>
+      </c>
+      <c r="M15" s="111">
         <v>1100</v>
       </c>
-      <c r="N15" s="113" t="s">
-        <v>275</v>
-      </c>
-      <c r="O15" s="114" t="s">
-        <v>276</v>
-      </c>
-      <c r="P15" s="114" t="s">
-        <v>276</v>
-      </c>
-      <c r="Q15" s="114">
+      <c r="N15" s="112" t="s">
+        <v>274</v>
+      </c>
+      <c r="O15" s="113">
+        <v>0.15809999999999999</v>
+      </c>
+      <c r="P15" s="68">
+        <f t="shared" si="0"/>
+        <v>17.865299999999998</v>
+      </c>
+      <c r="Q15" s="113">
         <v>0.15809999999999999</v>
       </c>
       <c r="R15" s="35">
         <f t="shared" si="1"/>
-        <v>18.971999999999998</v>
-      </c>
-      <c r="S15" s="114">
+        <v>17.865299999999998</v>
+      </c>
+      <c r="S15" s="113">
         <v>0.1177</v>
       </c>
       <c r="T15" s="35">
         <f t="shared" si="2"/>
         <v>129.47</v>
       </c>
-      <c r="U15" s="115"/>
+      <c r="U15" s="114"/>
       <c r="V15" s="21"/>
       <c r="W15" s="21"/>
     </row>
@@ -3107,7 +3097,7 @@
       <c r="A16" s="16">
         <v>14</v>
       </c>
-      <c r="B16" s="121"/>
+      <c r="B16" s="120"/>
       <c r="C16" s="71" t="s">
         <v>223</v>
       </c>
@@ -3145,25 +3135,25 @@
         <v>250</v>
       </c>
       <c r="O16" s="46">
-        <v>7.3099999999999998E-2</v>
+        <v>7.0300000000000001E-2</v>
       </c>
       <c r="P16" s="46">
         <f t="shared" si="0"/>
-        <v>0.73099999999999998</v>
+        <v>0.70300000000000007</v>
       </c>
       <c r="Q16" s="46">
-        <v>5.33E-2</v>
+        <v>5.1200000000000002E-2</v>
       </c>
       <c r="R16" s="46">
         <f t="shared" si="1"/>
-        <v>6.3959999999999999</v>
+        <v>6.1440000000000001</v>
       </c>
       <c r="S16" s="46">
-        <v>4.3700000000000003E-2</v>
+        <v>4.4200000000000003E-2</v>
       </c>
       <c r="T16" s="46">
         <f t="shared" si="2"/>
-        <v>48.07</v>
+        <v>48.620000000000005</v>
       </c>
       <c r="U16" s="26"/>
       <c r="V16" s="3"/>
@@ -3173,7 +3163,7 @@
       <c r="A17" s="16">
         <v>15</v>
       </c>
-      <c r="B17" s="120" t="s">
+      <c r="B17" s="119" t="s">
         <v>73</v>
       </c>
       <c r="C17" s="73" t="s">
@@ -3241,7 +3231,7 @@
       <c r="A18" s="16">
         <v>16</v>
       </c>
-      <c r="B18" s="120"/>
+      <c r="B18" s="119"/>
       <c r="C18" s="54" t="s">
         <v>124</v>
       </c>
@@ -3307,7 +3297,7 @@
       <c r="A19" s="16">
         <v>17</v>
       </c>
-      <c r="B19" s="119" t="s">
+      <c r="B19" s="118" t="s">
         <v>27</v>
       </c>
       <c r="C19" s="62" t="s">
@@ -3335,37 +3325,37 @@
         <v>1</v>
       </c>
       <c r="K19" s="66">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="L19" s="66">
-        <v>120</v>
+        <v>200</v>
       </c>
       <c r="M19" s="66">
         <v>1100</v>
       </c>
       <c r="N19" s="67" t="s">
-        <v>250</v>
+        <v>273</v>
       </c>
       <c r="O19" s="68">
-        <v>5.3699999999999998E-2</v>
+        <v>3.2300000000000002E-2</v>
       </c>
       <c r="P19" s="68">
         <f t="shared" si="0"/>
-        <v>1.0739999999999998</v>
+        <v>3.2300000000000004</v>
       </c>
       <c r="Q19" s="68">
-        <v>4.0599999999999997E-2</v>
+        <v>3.7400000000000003E-2</v>
       </c>
       <c r="R19" s="68">
         <f>Q19*L19</f>
-        <v>4.8719999999999999</v>
+        <v>7.48</v>
       </c>
       <c r="S19" s="68">
-        <v>3.5799999999999998E-2</v>
+        <v>2.9499999999999998E-2</v>
       </c>
       <c r="T19" s="68">
         <f t="shared" si="2"/>
-        <v>39.379999999999995</v>
+        <v>32.449999999999996</v>
       </c>
       <c r="U19" s="14"/>
       <c r="V19" s="3"/>
@@ -3375,12 +3365,12 @@
       <c r="A20" s="16">
         <v>18</v>
       </c>
-      <c r="B20" s="120"/>
+      <c r="B20" s="119"/>
       <c r="C20" s="28" t="s">
         <v>130</v>
       </c>
       <c r="D20" s="29" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="E20" s="29" t="s">
         <v>61</v>
@@ -3427,11 +3417,11 @@
         <v>4.9829999999999997</v>
       </c>
       <c r="S20" s="35">
-        <v>3.7499999999999999E-2</v>
+        <v>3.6299999999999999E-2</v>
       </c>
       <c r="T20" s="35">
         <f t="shared" si="2"/>
-        <v>41.25</v>
+        <v>39.93</v>
       </c>
       <c r="U20" s="15"/>
       <c r="V20" s="3"/>
@@ -3441,7 +3431,7 @@
       <c r="A21" s="16">
         <v>19</v>
       </c>
-      <c r="B21" s="121"/>
+      <c r="B21" s="120"/>
       <c r="C21" s="39" t="s">
         <v>131</v>
       </c>
@@ -3493,11 +3483,11 @@
         <v>13.632000000000001</v>
       </c>
       <c r="S21" s="46">
-        <v>8.0600000000000005E-2</v>
+        <v>0.1007</v>
       </c>
       <c r="T21" s="46">
         <f t="shared" si="2"/>
-        <v>88.660000000000011</v>
+        <v>110.77</v>
       </c>
       <c r="U21" s="82"/>
       <c r="V21" s="3"/>
@@ -3507,7 +3497,7 @@
       <c r="A22" s="16">
         <v>20</v>
       </c>
-      <c r="B22" s="119" t="s">
+      <c r="B22" s="118" t="s">
         <v>16</v>
       </c>
       <c r="C22" s="62" t="s">
@@ -3547,18 +3537,18 @@
         <v>250</v>
       </c>
       <c r="O22" s="68">
-        <v>1.4E-3</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="P22" s="68">
         <f t="shared" si="0"/>
-        <v>0.13999999999999999</v>
+        <v>0.12</v>
       </c>
       <c r="Q22" s="68">
-        <v>1.4E-3</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="R22" s="68">
         <f t="shared" si="1"/>
-        <v>0.84</v>
+        <v>0.72</v>
       </c>
       <c r="S22" s="68">
         <v>8.9999999999999998E-4</v>
@@ -3575,7 +3565,7 @@
       <c r="A23" s="16">
         <v>21</v>
       </c>
-      <c r="B23" s="120"/>
+      <c r="B23" s="119"/>
       <c r="C23" s="28" t="s">
         <v>138</v>
       </c>
@@ -3613,25 +3603,25 @@
         <v>250</v>
       </c>
       <c r="O23" s="35">
-        <v>1.4E-3</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="P23" s="35">
         <f>O23*K23</f>
-        <v>0.13999999999999999</v>
+        <v>0.11</v>
       </c>
       <c r="Q23" s="35">
-        <v>1.4E-3</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="R23" s="35">
         <f>L23*Q23</f>
-        <v>0.98</v>
+        <v>0.77</v>
       </c>
       <c r="S23" s="35">
-        <v>8.9999999999999998E-4</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="T23" s="35">
         <f t="shared" si="2"/>
-        <v>5.58</v>
+        <v>4.96</v>
       </c>
       <c r="U23" s="25"/>
       <c r="V23" s="3"/>
@@ -3641,7 +3631,7 @@
       <c r="A24" s="16">
         <v>22</v>
       </c>
-      <c r="B24" s="120"/>
+      <c r="B24" s="119"/>
       <c r="C24" s="28" t="s">
         <v>141</v>
       </c>
@@ -3707,7 +3697,7 @@
       <c r="A25" s="16">
         <v>23</v>
       </c>
-      <c r="B25" s="120"/>
+      <c r="B25" s="119"/>
       <c r="C25" s="28" t="s">
         <v>143</v>
       </c>
@@ -3745,25 +3735,25 @@
         <v>250</v>
       </c>
       <c r="O25" s="35">
-        <v>1.2999999999999999E-3</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="P25" s="35">
         <f t="shared" si="0"/>
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="Q25" s="35">
-        <v>1.2999999999999999E-3</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="R25" s="35">
         <f t="shared" si="1"/>
-        <v>0.26</v>
+        <v>0.22</v>
       </c>
       <c r="S25" s="35">
-        <v>8.9999999999999998E-4</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="T25" s="35">
         <f t="shared" si="2"/>
-        <v>0.99</v>
+        <v>0.88</v>
       </c>
       <c r="U25" s="36"/>
       <c r="V25" s="3"/>
@@ -3773,7 +3763,7 @@
       <c r="A26" s="16">
         <v>24</v>
       </c>
-      <c r="B26" s="120"/>
+      <c r="B26" s="119"/>
       <c r="C26" s="28" t="s">
         <v>145</v>
       </c>
@@ -3839,7 +3829,7 @@
       <c r="A27" s="16">
         <v>25</v>
       </c>
-      <c r="B27" s="120"/>
+      <c r="B27" s="119"/>
       <c r="C27" s="28" t="s">
         <v>148</v>
       </c>
@@ -3905,7 +3895,7 @@
       <c r="A28" s="16">
         <v>26</v>
       </c>
-      <c r="B28" s="120"/>
+      <c r="B28" s="119"/>
       <c r="C28" s="28" t="s">
         <v>152</v>
       </c>
@@ -3950,11 +3940,11 @@
         <v>0.42</v>
       </c>
       <c r="Q28" s="35">
-        <v>6.1999999999999998E-3</v>
+        <v>8.3999999999999995E-3</v>
       </c>
       <c r="R28" s="35">
         <f t="shared" si="1"/>
-        <v>0.92999999999999994</v>
+        <v>1.26</v>
       </c>
       <c r="S28" s="35">
         <v>6.1999999999999998E-3</v>
@@ -3971,7 +3961,7 @@
       <c r="A29" s="16">
         <v>27</v>
       </c>
-      <c r="B29" s="120"/>
+      <c r="B29" s="119"/>
       <c r="C29" s="70" t="s">
         <v>229</v>
       </c>
@@ -4037,7 +4027,7 @@
       <c r="A30" s="16">
         <v>28</v>
       </c>
-      <c r="B30" s="120"/>
+      <c r="B30" s="119"/>
       <c r="C30" s="28" t="s">
         <v>155</v>
       </c>
@@ -4075,25 +4065,25 @@
         <v>250</v>
       </c>
       <c r="O30" s="35">
-        <v>1.6999999999999999E-3</v>
+        <v>1.4E-3</v>
       </c>
       <c r="P30" s="35">
         <f t="shared" si="0"/>
-        <v>0.16999999999999998</v>
+        <v>0.13999999999999999</v>
       </c>
       <c r="Q30" s="35">
-        <v>1.6999999999999999E-3</v>
+        <v>1.4E-3</v>
       </c>
       <c r="R30" s="35">
         <f t="shared" si="1"/>
-        <v>0.67999999999999994</v>
+        <v>0.55999999999999994</v>
       </c>
       <c r="S30" s="35">
-        <v>1.2999999999999999E-3</v>
+        <v>1.1000000000000001E-3</v>
       </c>
       <c r="T30" s="35">
         <f t="shared" si="2"/>
-        <v>4.03</v>
+        <v>3.41</v>
       </c>
       <c r="U30" s="25"/>
       <c r="V30" s="3"/>
@@ -4103,7 +4093,7 @@
       <c r="A31" s="16">
         <v>29</v>
       </c>
-      <c r="B31" s="120"/>
+      <c r="B31" s="119"/>
       <c r="C31" s="28" t="s">
         <v>158</v>
       </c>
@@ -4141,69 +4131,67 @@
         <v>250</v>
       </c>
       <c r="O31" s="35">
-        <v>2.0999999999999999E-3</v>
+        <v>1.5E-3</v>
       </c>
       <c r="P31" s="35">
         <f t="shared" si="0"/>
-        <v>0.21</v>
+        <v>0.15</v>
       </c>
       <c r="Q31" s="35">
-        <v>2.0999999999999999E-3</v>
+        <v>1.5E-3</v>
       </c>
       <c r="R31" s="35">
         <f t="shared" si="1"/>
-        <v>0.42</v>
+        <v>0.3</v>
       </c>
       <c r="S31" s="35">
-        <v>1.6999999999999999E-3</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="T31" s="35">
         <f t="shared" si="2"/>
-        <v>1.8699999999999999</v>
+        <v>1.3199999999999998</v>
       </c>
       <c r="U31" s="25"/>
       <c r="V31" s="3"/>
       <c r="W31" s="3"/>
     </row>
-    <row r="32" spans="1:23" s="125" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" s="116" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="16">
         <v>30</v>
       </c>
-      <c r="B32" s="120"/>
+      <c r="B32" s="119"/>
       <c r="C32" s="70" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="D32" s="31" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="E32" s="31" t="s">
         <v>136</v>
       </c>
       <c r="F32" s="31" t="s">
+        <v>283</v>
+      </c>
+      <c r="G32" s="30" t="s">
         <v>285</v>
       </c>
-      <c r="G32" s="30" t="s">
-        <v>287</v>
-      </c>
       <c r="H32" s="29" t="s">
         <v>219</v>
       </c>
       <c r="I32" s="31" t="s">
-        <v>286</v>
-      </c>
-      <c r="J32" s="102">
+        <v>284</v>
+      </c>
+      <c r="J32" s="101">
         <v>8</v>
       </c>
       <c r="K32" s="33">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="L32" s="33">
-        <f>J32*100</f>
-        <v>800</v>
+        <v>830</v>
       </c>
       <c r="M32" s="33">
-        <f>J32*1000</f>
-        <v>8000</v>
+        <v>8200</v>
       </c>
       <c r="N32" s="34" t="s">
         <v>250</v>
@@ -4213,31 +4201,31 @@
       </c>
       <c r="P32" s="35">
         <f t="shared" si="0"/>
-        <v>1.4000000000000001</v>
+        <v>1.7500000000000002</v>
       </c>
       <c r="Q32" s="35">
         <v>2.5600000000000001E-2</v>
       </c>
       <c r="R32" s="35">
         <f>Q32*L32</f>
-        <v>20.48</v>
+        <v>21.248000000000001</v>
       </c>
       <c r="S32" s="35">
         <v>2.35E-2</v>
       </c>
       <c r="T32" s="35">
         <f>S32*M32</f>
-        <v>188</v>
+        <v>192.7</v>
       </c>
       <c r="U32" s="25"/>
-      <c r="V32" s="124"/>
-      <c r="W32" s="124"/>
+      <c r="V32" s="115"/>
+      <c r="W32" s="115"/>
     </row>
     <row r="33" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="16">
         <v>31</v>
       </c>
-      <c r="B33" s="120"/>
+      <c r="B33" s="119"/>
       <c r="C33" s="70" t="s">
         <v>230</v>
       </c>
@@ -4263,7 +4251,7 @@
         <v>1</v>
       </c>
       <c r="K33" s="33">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="L33" s="33">
         <v>120</v>
@@ -4279,7 +4267,7 @@
       </c>
       <c r="P33" s="35">
         <f t="shared" si="0"/>
-        <v>0.71400000000000008</v>
+        <v>0.35700000000000004</v>
       </c>
       <c r="Q33" s="35">
         <v>2.75E-2</v>
@@ -4303,7 +4291,7 @@
       <c r="A34" s="16">
         <v>32</v>
       </c>
-      <c r="B34" s="120"/>
+      <c r="B34" s="119"/>
       <c r="C34" s="28" t="s">
         <v>162</v>
       </c>
@@ -4369,7 +4357,7 @@
       <c r="A35" s="16">
         <v>33</v>
       </c>
-      <c r="B35" s="121"/>
+      <c r="B35" s="120"/>
       <c r="C35" s="39" t="s">
         <v>165</v>
       </c>
@@ -4395,7 +4383,7 @@
         <v>4</v>
       </c>
       <c r="K35" s="44">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="K11:K50" si="3">J35*5</f>
         <v>20</v>
       </c>
       <c r="L35" s="44">
@@ -4436,7 +4424,7 @@
       <c r="A36" s="16">
         <v>34</v>
       </c>
-      <c r="B36" s="120" t="s">
+      <c r="B36" s="119" t="s">
         <v>74</v>
       </c>
       <c r="C36" s="73" t="s">
@@ -4460,7 +4448,7 @@
       <c r="I36" s="85" t="s">
         <v>219</v>
       </c>
-      <c r="J36" s="86">
+      <c r="J36" s="49">
         <v>1</v>
       </c>
       <c r="K36" s="49">
@@ -4476,25 +4464,25 @@
         <v>250</v>
       </c>
       <c r="O36" s="51">
-        <v>5.1799999999999999E-2</v>
+        <v>2.5899999999999999E-2</v>
       </c>
       <c r="P36" s="51">
         <f t="shared" si="0"/>
-        <v>0.51800000000000002</v>
+        <v>0.25900000000000001</v>
       </c>
       <c r="Q36" s="51">
-        <v>3.7400000000000003E-2</v>
+        <v>1.8700000000000001E-2</v>
       </c>
       <c r="R36" s="51">
         <f t="shared" si="1"/>
-        <v>4.4880000000000004</v>
+        <v>2.2440000000000002</v>
       </c>
       <c r="S36" s="51">
-        <v>1.29E-2</v>
+        <v>1.61E-2</v>
       </c>
       <c r="T36" s="51">
         <f t="shared" si="2"/>
-        <v>14.19</v>
+        <v>17.71</v>
       </c>
       <c r="U36" s="52"/>
       <c r="V36" s="3"/>
@@ -4504,8 +4492,8 @@
       <c r="A37" s="16">
         <v>35</v>
       </c>
-      <c r="B37" s="120"/>
-      <c r="C37" s="87" t="s">
+      <c r="B37" s="119"/>
+      <c r="C37" s="86" t="s">
         <v>231</v>
       </c>
       <c r="D37" s="55" t="s">
@@ -4526,11 +4514,11 @@
       <c r="I37" s="55" t="s">
         <v>219</v>
       </c>
-      <c r="J37" s="88">
+      <c r="J37" s="87">
         <v>1</v>
       </c>
       <c r="K37" s="58">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L37" s="58">
         <v>120</v>
@@ -4542,25 +4530,25 @@
         <v>250</v>
       </c>
       <c r="O37" s="60">
-        <v>0.1308</v>
+        <v>0.10521</v>
       </c>
       <c r="P37" s="60">
         <f t="shared" si="0"/>
-        <v>1.3080000000000001</v>
+        <v>0.73646999999999996</v>
       </c>
       <c r="Q37" s="60">
-        <v>9.5200000000000007E-2</v>
+        <v>8.4168000000000007E-2</v>
       </c>
       <c r="R37" s="60">
         <f t="shared" si="1"/>
-        <v>11.424000000000001</v>
+        <v>10.100160000000001</v>
       </c>
       <c r="S37" s="60">
-        <v>8.2100000000000006E-2</v>
+        <v>7.7154E-2</v>
       </c>
       <c r="T37" s="60">
         <f t="shared" si="2"/>
-        <v>90.31</v>
+        <v>84.869399999999999</v>
       </c>
       <c r="U37" s="61"/>
       <c r="V37" s="3"/>
@@ -4570,7 +4558,7 @@
       <c r="A38" s="16">
         <v>36</v>
       </c>
-      <c r="B38" s="119" t="s">
+      <c r="B38" s="118" t="s">
         <v>75</v>
       </c>
       <c r="C38" s="62" t="s">
@@ -4607,14 +4595,14 @@
         <v>1020</v>
       </c>
       <c r="N38" s="67" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="O38" s="68">
-        <v>2.8319999999999999</v>
+        <v>3.3984000000000001</v>
       </c>
       <c r="P38" s="68">
         <f t="shared" si="0"/>
-        <v>19.823999999999998</v>
+        <v>23.788800000000002</v>
       </c>
       <c r="Q38" s="68">
         <v>1.8691199999999999</v>
@@ -4630,7 +4618,7 @@
         <f t="shared" si="2"/>
         <v>1733.184</v>
       </c>
-      <c r="U38" s="89"/>
+      <c r="U38" s="88"/>
       <c r="V38" s="3"/>
       <c r="W38" s="3"/>
     </row>
@@ -4638,7 +4626,7 @@
       <c r="A39" s="16">
         <v>37</v>
       </c>
-      <c r="B39" s="120"/>
+      <c r="B39" s="119"/>
       <c r="C39" s="28" t="s">
         <v>182</v>
       </c>
@@ -4676,25 +4664,25 @@
         <v>250</v>
       </c>
       <c r="O39" s="35">
-        <v>0.37019999999999997</v>
+        <v>0.33729999999999999</v>
       </c>
       <c r="P39" s="35">
         <f t="shared" si="0"/>
-        <v>2.5913999999999997</v>
+        <v>2.3611</v>
       </c>
       <c r="Q39" s="35">
-        <v>0.25190000000000001</v>
+        <v>0.21099999999999999</v>
       </c>
       <c r="R39" s="35">
         <f t="shared" si="1"/>
-        <v>26.4495</v>
+        <v>22.154999999999998</v>
       </c>
       <c r="S39" s="35">
-        <v>0.24160000000000001</v>
+        <v>0.20019999999999999</v>
       </c>
       <c r="T39" s="35">
         <f t="shared" si="2"/>
-        <v>246.43200000000002</v>
+        <v>204.20399999999998</v>
       </c>
       <c r="U39" s="25"/>
       <c r="V39" s="3"/>
@@ -4704,7 +4692,7 @@
       <c r="A40" s="16">
         <v>38</v>
       </c>
-      <c r="B40" s="120"/>
+      <c r="B40" s="119"/>
       <c r="C40" s="70" t="s">
         <v>235</v>
       </c>
@@ -4730,16 +4718,13 @@
         <v>1</v>
       </c>
       <c r="K40" s="33">
-        <f t="shared" si="3"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L40" s="33">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="M40" s="33">
-        <f t="shared" si="5"/>
-        <v>1000</v>
+        <v>1020</v>
       </c>
       <c r="N40" s="34" t="s">
         <v>17</v>
@@ -4749,21 +4734,21 @@
       </c>
       <c r="P40" s="35">
         <f t="shared" si="0"/>
-        <v>2.4</v>
+        <v>3.36</v>
       </c>
       <c r="Q40" s="35">
         <v>0.2656</v>
       </c>
       <c r="R40" s="35">
         <f t="shared" si="1"/>
-        <v>26.56</v>
+        <v>27.888000000000002</v>
       </c>
       <c r="S40" s="35">
         <v>0.14940000000000001</v>
       </c>
       <c r="T40" s="35">
         <f t="shared" si="2"/>
-        <v>149.4</v>
+        <v>152.38800000000001</v>
       </c>
       <c r="U40" s="25"/>
       <c r="V40" s="3"/>
@@ -4773,7 +4758,7 @@
       <c r="A41" s="16">
         <v>39</v>
       </c>
-      <c r="B41" s="120"/>
+      <c r="B41" s="119"/>
       <c r="C41" s="28" t="s">
         <v>186</v>
       </c>
@@ -4799,40 +4784,37 @@
         <v>1</v>
       </c>
       <c r="K41" s="33">
-        <f t="shared" si="3"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L41" s="33">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="M41" s="33">
-        <f t="shared" si="5"/>
-        <v>1000</v>
+        <v>1020</v>
       </c>
       <c r="N41" s="34" t="s">
         <v>17</v>
       </c>
       <c r="O41" s="35">
-        <v>0.67</v>
+        <v>0.81</v>
       </c>
       <c r="P41" s="35">
         <f t="shared" si="0"/>
-        <v>3.35</v>
+        <v>5.67</v>
       </c>
       <c r="Q41" s="35">
-        <v>0.45290000000000002</v>
+        <v>0.54400000000000004</v>
       </c>
       <c r="R41" s="35">
         <f t="shared" si="1"/>
-        <v>45.29</v>
+        <v>57.120000000000005</v>
       </c>
       <c r="S41" s="35">
-        <v>0.28639999999999999</v>
+        <v>0.34399999999999997</v>
       </c>
       <c r="T41" s="35">
         <f t="shared" si="2"/>
-        <v>286.39999999999998</v>
+        <v>350.88</v>
       </c>
       <c r="U41" s="25"/>
       <c r="V41" s="3"/>
@@ -4842,7 +4824,7 @@
       <c r="A42" s="16">
         <v>40</v>
       </c>
-      <c r="B42" s="120"/>
+      <c r="B42" s="119"/>
       <c r="C42" s="70" t="s">
         <v>240</v>
       </c>
@@ -4868,40 +4850,37 @@
         <v>1</v>
       </c>
       <c r="K42" s="33">
-        <f t="shared" si="3"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L42" s="33">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="M42" s="33">
-        <f t="shared" si="5"/>
-        <v>1000</v>
+        <v>1020</v>
       </c>
       <c r="N42" s="34" t="s">
-        <v>250</v>
+        <v>286</v>
       </c>
       <c r="O42" s="35">
-        <v>8.8099999999999998E-2</v>
+        <v>5.1299999999999998E-2</v>
       </c>
       <c r="P42" s="35">
         <f t="shared" si="0"/>
-        <v>0.4405</v>
+        <v>0.35909999999999997</v>
       </c>
       <c r="Q42" s="35">
-        <v>6.7299999999999999E-2</v>
+        <v>0.05</v>
       </c>
       <c r="R42" s="35">
         <f t="shared" si="1"/>
-        <v>6.7299999999999995</v>
+        <v>5.25</v>
       </c>
       <c r="S42" s="35">
-        <v>5.0700000000000002E-2</v>
+        <v>0.05</v>
       </c>
       <c r="T42" s="35">
         <f t="shared" si="2"/>
-        <v>50.7</v>
+        <v>51</v>
       </c>
       <c r="U42" s="15"/>
       <c r="V42" s="3"/>
@@ -4911,7 +4890,7 @@
       <c r="A43" s="16">
         <v>41</v>
       </c>
-      <c r="B43" s="120"/>
+      <c r="B43" s="119"/>
       <c r="C43" s="70" t="s">
         <v>71</v>
       </c>
@@ -4937,40 +4916,37 @@
         <v>1</v>
       </c>
       <c r="K43" s="33">
-        <f t="shared" si="3"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L43" s="33">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="M43" s="33">
-        <f t="shared" si="5"/>
-        <v>1000</v>
+        <v>1020</v>
       </c>
       <c r="N43" s="34" t="s">
         <v>233</v>
       </c>
       <c r="O43" s="35">
-        <v>0.51</v>
+        <v>0.51300000000000001</v>
       </c>
       <c r="P43" s="35">
         <f t="shared" si="0"/>
-        <v>2.5499999999999998</v>
+        <v>3.5910000000000002</v>
       </c>
       <c r="Q43" s="35">
         <v>0.30599999999999999</v>
       </c>
       <c r="R43" s="35">
         <f t="shared" si="1"/>
-        <v>30.599999999999998</v>
+        <v>32.130000000000003</v>
       </c>
       <c r="S43" s="35">
-        <v>0.25900000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="T43" s="35">
         <f t="shared" si="2"/>
-        <v>259</v>
+        <v>204</v>
       </c>
       <c r="U43" s="25"/>
       <c r="V43" s="3"/>
@@ -4980,7 +4956,7 @@
       <c r="A44" s="16">
         <v>42</v>
       </c>
-      <c r="B44" s="120"/>
+      <c r="B44" s="119"/>
       <c r="C44" s="70" t="s">
         <v>243</v>
       </c>
@@ -5006,43 +4982,40 @@
         <v>1</v>
       </c>
       <c r="K44" s="33">
-        <f t="shared" si="3"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L44" s="33">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="M44" s="33">
-        <f t="shared" si="5"/>
-        <v>1000</v>
+        <v>1020</v>
       </c>
       <c r="N44" s="34" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="O44" s="35">
-        <v>1.45</v>
+        <v>6</v>
       </c>
       <c r="P44" s="35">
         <f t="shared" si="0"/>
-        <v>7.25</v>
+        <v>42</v>
       </c>
       <c r="Q44" s="35">
-        <v>1.1000000000000001</v>
+        <v>6</v>
       </c>
       <c r="R44" s="35">
         <f t="shared" si="1"/>
-        <v>110.00000000000001</v>
+        <v>630</v>
       </c>
       <c r="S44" s="35">
-        <v>0.77</v>
+        <v>6</v>
       </c>
       <c r="T44" s="35">
         <f t="shared" si="2"/>
-        <v>770</v>
+        <v>6120</v>
       </c>
       <c r="U44" s="36" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="V44" s="3"/>
       <c r="W44" s="3"/>
@@ -5051,7 +5024,7 @@
       <c r="A45" s="16">
         <v>43</v>
       </c>
-      <c r="B45" s="120"/>
+      <c r="B45" s="119"/>
       <c r="C45" s="70" t="s">
         <v>247</v>
       </c>
@@ -5077,40 +5050,37 @@
         <v>1</v>
       </c>
       <c r="K45" s="33">
-        <f t="shared" si="3"/>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L45" s="33">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="M45" s="33">
-        <f t="shared" si="5"/>
-        <v>1000</v>
+        <v>1020</v>
       </c>
       <c r="N45" s="34" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="O45" s="35">
-        <v>1.88</v>
+        <v>2.4249999999999998</v>
       </c>
       <c r="P45" s="35">
         <f t="shared" si="0"/>
-        <v>9.3999999999999986</v>
+        <v>24.25</v>
       </c>
       <c r="Q45" s="35">
-        <v>1.88</v>
+        <v>2.1272727272727199</v>
       </c>
       <c r="R45" s="35">
         <f t="shared" si="1"/>
-        <v>188</v>
+        <v>233.99999999999918</v>
       </c>
       <c r="S45" s="35">
-        <v>1.88</v>
+        <v>2.0401960784313702</v>
       </c>
       <c r="T45" s="35">
         <f t="shared" si="2"/>
-        <v>1880</v>
+        <v>2080.9999999999977</v>
       </c>
       <c r="U45" s="36"/>
       <c r="V45" s="3"/>
@@ -5120,7 +5090,7 @@
       <c r="A46" s="16">
         <v>44</v>
       </c>
-      <c r="B46" s="121"/>
+      <c r="B46" s="120"/>
       <c r="C46" s="39" t="s">
         <v>191</v>
       </c>
@@ -5146,42 +5116,39 @@
         <v>1</v>
       </c>
       <c r="K46" s="44">
-        <f t="shared" si="3"/>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L46" s="44">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="M46" s="44">
-        <f t="shared" si="5"/>
-        <v>1000</v>
+        <v>1020</v>
       </c>
       <c r="N46" s="45" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="O46" s="46">
-        <v>0.22559999999999999</v>
+        <v>1.1160000000000001</v>
       </c>
       <c r="P46" s="46">
         <f t="shared" si="0"/>
-        <v>1.1279999999999999</v>
+        <v>11.16</v>
       </c>
       <c r="Q46" s="46">
-        <v>0.22559999999999999</v>
+        <v>1.06</v>
       </c>
       <c r="R46" s="46">
         <f>Q46*L46</f>
-        <v>22.56</v>
+        <v>116.60000000000001</v>
       </c>
       <c r="S46" s="46">
-        <v>0.22559999999999999</v>
+        <v>1.0598039215686199</v>
       </c>
       <c r="T46" s="46">
         <f t="shared" si="2"/>
-        <v>225.6</v>
-      </c>
-      <c r="U46" s="90"/>
+        <v>1080.9999999999923</v>
+      </c>
+      <c r="U46" s="89"/>
       <c r="V46" s="3"/>
       <c r="W46" s="3"/>
     </row>
@@ -5189,10 +5156,10 @@
       <c r="A47" s="16">
         <v>45</v>
       </c>
-      <c r="B47" s="110" t="s">
+      <c r="B47" s="109" t="s">
         <v>248</v>
       </c>
-      <c r="C47" s="91" t="s">
+      <c r="C47" s="90" t="s">
         <v>194</v>
       </c>
       <c r="D47" s="85" t="s">
@@ -5207,52 +5174,49 @@
       <c r="G47" s="85" t="s">
         <v>261</v>
       </c>
-      <c r="H47" s="92" t="s">
+      <c r="H47" s="91" t="s">
         <v>262</v>
       </c>
-      <c r="I47" s="92" t="s">
+      <c r="I47" s="91" t="s">
         <v>263</v>
       </c>
-      <c r="J47" s="93">
+      <c r="J47" s="92">
         <v>1</v>
       </c>
-      <c r="K47" s="94">
-        <f t="shared" si="3"/>
-        <v>5</v>
-      </c>
-      <c r="L47" s="94">
-        <f t="shared" si="4"/>
-        <v>100</v>
-      </c>
-      <c r="M47" s="94">
-        <f t="shared" si="5"/>
-        <v>1000</v>
-      </c>
-      <c r="N47" s="95" t="s">
+      <c r="K47" s="93">
+        <v>7</v>
+      </c>
+      <c r="L47" s="93">
+        <v>105</v>
+      </c>
+      <c r="M47" s="93">
+        <v>1020</v>
+      </c>
+      <c r="N47" s="94" t="s">
         <v>250</v>
       </c>
-      <c r="O47" s="96">
+      <c r="O47" s="95">
         <v>0.28570000000000001</v>
       </c>
-      <c r="P47" s="96">
+      <c r="P47" s="95">
         <f t="shared" si="0"/>
-        <v>1.4285000000000001</v>
-      </c>
-      <c r="Q47" s="96">
+        <v>1.9999</v>
+      </c>
+      <c r="Q47" s="95">
         <v>0.1459</v>
       </c>
-      <c r="R47" s="96">
+      <c r="R47" s="95">
         <f t="shared" si="1"/>
-        <v>14.59</v>
-      </c>
-      <c r="S47" s="96">
+        <v>15.3195</v>
+      </c>
+      <c r="S47" s="95">
         <v>0.13980000000000001</v>
       </c>
-      <c r="T47" s="96">
+      <c r="T47" s="95">
         <f t="shared" si="2"/>
-        <v>139.80000000000001</v>
-      </c>
-      <c r="U47" s="97"/>
+        <v>142.596</v>
+      </c>
+      <c r="U47" s="96"/>
       <c r="V47" s="3"/>
       <c r="W47" s="3"/>
     </row>
@@ -5260,7 +5224,7 @@
       <c r="A48" s="16">
         <v>46</v>
       </c>
-      <c r="B48" s="119" t="s">
+      <c r="B48" s="118" t="s">
         <v>76</v>
       </c>
       <c r="C48" s="62" t="s">
@@ -5288,43 +5252,40 @@
         <v>1</v>
       </c>
       <c r="K48" s="66">
-        <f t="shared" si="3"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="L48" s="66">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="M48" s="66">
-        <f t="shared" si="5"/>
-        <v>1000</v>
-      </c>
-      <c r="N48" s="98" t="s">
+        <v>1020</v>
+      </c>
+      <c r="N48" s="97" t="s">
         <v>250</v>
       </c>
-      <c r="O48" s="99">
+      <c r="O48" s="98">
         <v>0.74480000000000002</v>
       </c>
       <c r="P48" s="68">
         <f t="shared" si="0"/>
-        <v>3.7240000000000002</v>
-      </c>
-      <c r="Q48" s="99">
-        <v>0.41560000000000002</v>
+        <v>5.2136000000000005</v>
+      </c>
+      <c r="Q48" s="98">
+        <v>0.44330000000000003</v>
       </c>
       <c r="R48" s="68">
         <f t="shared" si="1"/>
-        <v>41.56</v>
+        <v>46.546500000000002</v>
       </c>
       <c r="S48" s="68">
-        <v>0.39279999999999998</v>
+        <v>0.41899999999999998</v>
       </c>
       <c r="T48" s="68">
         <f t="shared" si="2"/>
-        <v>392.79999999999995</v>
-      </c>
-      <c r="U48" s="89" t="s">
-        <v>281</v>
+        <v>427.38</v>
+      </c>
+      <c r="U48" s="88" t="s">
+        <v>279</v>
       </c>
       <c r="V48" s="3"/>
       <c r="W48" s="3"/>
@@ -5333,7 +5294,7 @@
       <c r="A49" s="16">
         <v>47</v>
       </c>
-      <c r="B49" s="120"/>
+      <c r="B49" s="119"/>
       <c r="C49" s="28" t="s">
         <v>198</v>
       </c>
@@ -5355,22 +5316,19 @@
       <c r="I49" s="29" t="s">
         <v>219</v>
       </c>
-      <c r="J49" s="100">
+      <c r="J49" s="99">
         <v>2</v>
       </c>
       <c r="K49" s="33">
-        <f t="shared" si="3"/>
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="L49" s="33">
-        <f t="shared" si="4"/>
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="M49" s="33">
-        <f t="shared" si="5"/>
-        <v>2000</v>
-      </c>
-      <c r="N49" s="101" t="s">
+        <v>2020</v>
+      </c>
+      <c r="N49" s="100" t="s">
         <v>250</v>
       </c>
       <c r="O49" s="35">
@@ -5378,21 +5336,21 @@
       </c>
       <c r="P49" s="35">
         <f t="shared" si="0"/>
-        <v>0.44699999999999995</v>
+        <v>0.89399999999999991</v>
       </c>
       <c r="Q49" s="35">
         <v>3.39E-2</v>
       </c>
       <c r="R49" s="35">
         <f t="shared" si="1"/>
-        <v>6.78</v>
+        <v>7.1189999999999998</v>
       </c>
       <c r="S49" s="35">
-        <v>2.4E-2</v>
+        <v>2.9899999999999999E-2</v>
       </c>
       <c r="T49" s="35">
         <f t="shared" si="2"/>
-        <v>48</v>
+        <v>60.397999999999996</v>
       </c>
       <c r="U49" s="25"/>
       <c r="V49" s="3"/>
@@ -5402,7 +5360,7 @@
       <c r="A50" s="16">
         <v>48</v>
       </c>
-      <c r="B50" s="120"/>
+      <c r="B50" s="119"/>
       <c r="C50" s="28" t="s">
         <v>201</v>
       </c>
@@ -5424,22 +5382,19 @@
       <c r="I50" s="29" t="s">
         <v>219</v>
       </c>
-      <c r="J50" s="102">
+      <c r="J50" s="101">
         <v>1</v>
       </c>
       <c r="K50" s="33">
-        <f t="shared" si="3"/>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="L50" s="33">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="M50" s="33">
-        <f t="shared" si="5"/>
-        <v>1000</v>
-      </c>
-      <c r="N50" s="101" t="s">
+        <v>1020</v>
+      </c>
+      <c r="N50" s="100" t="s">
         <v>250</v>
       </c>
       <c r="O50" s="35">
@@ -5447,23 +5402,23 @@
       </c>
       <c r="P50" s="35">
         <f t="shared" si="0"/>
-        <v>0.58250000000000002</v>
+        <v>1.165</v>
       </c>
       <c r="Q50" s="35">
         <v>8.4099999999999994E-2</v>
       </c>
       <c r="R50" s="35">
         <f t="shared" si="1"/>
-        <v>8.41</v>
+        <v>9.2509999999999994</v>
       </c>
       <c r="S50" s="35">
-        <v>3.61E-2</v>
+        <v>6.9400000000000003E-2</v>
       </c>
       <c r="T50" s="35">
         <f t="shared" si="2"/>
-        <v>36.1</v>
-      </c>
-      <c r="U50" s="103"/>
+        <v>70.787999999999997</v>
+      </c>
+      <c r="U50" s="102"/>
       <c r="V50" s="3"/>
       <c r="W50" s="3"/>
     </row>
@@ -5471,7 +5426,7 @@
       <c r="A51" s="16">
         <v>49</v>
       </c>
-      <c r="B51" s="120"/>
+      <c r="B51" s="119"/>
       <c r="C51" s="28" t="s">
         <v>204</v>
       </c>
@@ -5493,54 +5448,51 @@
       <c r="I51" s="29" t="s">
         <v>219</v>
       </c>
-      <c r="J51" s="102">
+      <c r="J51" s="101">
         <v>1</v>
       </c>
       <c r="K51" s="33">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="L51" s="33">
-        <f t="shared" si="4"/>
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="M51" s="33">
-        <v>200</v>
-      </c>
-      <c r="N51" s="101" t="s">
-        <v>273</v>
+        <v>1020</v>
+      </c>
+      <c r="N51" s="100" t="s">
+        <v>250</v>
       </c>
       <c r="O51" s="35">
-        <v>7.6999999999999999E-2</v>
+        <v>5.4899999999999997E-2</v>
       </c>
       <c r="P51" s="35">
         <f t="shared" si="0"/>
-        <v>7.7</v>
+        <v>0.54899999999999993</v>
       </c>
       <c r="Q51" s="35">
-        <v>7.6999999999999999E-2</v>
+        <v>4.0500000000000001E-2</v>
       </c>
       <c r="R51" s="35">
         <f t="shared" si="1"/>
-        <v>7.7</v>
+        <v>4.4550000000000001</v>
       </c>
       <c r="S51" s="35">
-        <v>7.6999999999999999E-2</v>
+        <v>3.5200000000000002E-2</v>
       </c>
       <c r="T51" s="35">
         <f t="shared" si="2"/>
-        <v>15.4</v>
-      </c>
-      <c r="U51" s="36" t="s">
-        <v>274</v>
-      </c>
+        <v>35.904000000000003</v>
+      </c>
+      <c r="U51" s="36"/>
       <c r="V51" s="3"/>
       <c r="W51" s="3"/>
     </row>
     <row r="52" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="126">
+      <c r="A52" s="117">
         <v>50</v>
       </c>
-      <c r="B52" s="121"/>
+      <c r="B52" s="120"/>
       <c r="C52" s="39" t="s">
         <v>208</v>
       </c>
@@ -5562,90 +5514,90 @@
       <c r="I52" s="40" t="s">
         <v>219</v>
       </c>
-      <c r="J52" s="104">
+      <c r="J52" s="103">
         <v>1</v>
       </c>
       <c r="K52" s="44">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L52" s="44">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="M52" s="44">
-        <v>1050</v>
-      </c>
-      <c r="N52" s="105" t="s">
-        <v>250</v>
+        <v>1020</v>
+      </c>
+      <c r="N52" s="104" t="s">
+        <v>287</v>
       </c>
       <c r="O52" s="46">
-        <v>0.1085</v>
-      </c>
-      <c r="P52" s="106">
+        <v>0.2</v>
+      </c>
+      <c r="P52" s="105">
         <f t="shared" si="0"/>
-        <v>1.085</v>
+        <v>1.4000000000000001</v>
       </c>
       <c r="Q52" s="46">
-        <v>8.0799999999999997E-2</v>
+        <v>0.2</v>
       </c>
       <c r="R52" s="46">
         <f t="shared" si="1"/>
-        <v>9.6959999999999997</v>
+        <v>22</v>
       </c>
       <c r="S52" s="46">
-        <v>6.2199999999999998E-2</v>
+        <v>0.2</v>
       </c>
       <c r="T52" s="46">
         <f t="shared" si="2"/>
-        <v>65.31</v>
+        <v>204</v>
       </c>
       <c r="U52" s="26"/>
       <c r="V52" s="3"/>
       <c r="W52" s="3"/>
     </row>
     <row r="53" spans="1:23" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="K53" s="122" t="s">
+      <c r="K53" s="121" t="s">
         <v>18</v>
       </c>
-      <c r="L53" s="122"/>
-      <c r="M53" s="122"/>
-      <c r="N53" s="122"/>
+      <c r="L53" s="121"/>
+      <c r="M53" s="121"/>
+      <c r="N53" s="121"/>
       <c r="P53" s="17">
         <f>SUM(P3:P52)</f>
-        <v>109.74689999999998</v>
+        <v>192.83976999999999</v>
       </c>
       <c r="Q53" s="7"/>
       <c r="R53" s="17">
         <f>SUM(R3:R52)</f>
-        <v>987.14509999999996</v>
+        <v>1674.4620599999989</v>
       </c>
       <c r="S53" s="8"/>
       <c r="T53" s="17">
         <f>SUM(T3:T52)</f>
-        <v>7910.8860000000013</v>
+        <v>14790.281399999991</v>
       </c>
       <c r="V53" s="3"/>
       <c r="W53" s="3"/>
     </row>
     <row r="54" spans="1:23" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K54" s="123" t="s">
+      <c r="K54" s="122" t="s">
         <v>19</v>
       </c>
-      <c r="L54" s="123"/>
-      <c r="M54" s="123"/>
-      <c r="N54" s="123"/>
+      <c r="L54" s="122"/>
+      <c r="M54" s="122"/>
+      <c r="N54" s="122"/>
       <c r="P54" s="27">
         <f>P53/5</f>
-        <v>21.949379999999998</v>
+        <v>38.567954</v>
       </c>
       <c r="Q54" s="8"/>
       <c r="R54" s="9">
         <f>R53/100</f>
-        <v>9.8714510000000004</v>
+        <v>16.74462059999999</v>
       </c>
       <c r="S54" s="9"/>
       <c r="T54" s="9">
         <f>T53/1000</f>
-        <v>7.9108860000000014</v>
+        <v>14.790281399999991</v>
       </c>
       <c r="V54" s="3"/>
       <c r="W54" s="3"/>
@@ -5684,6 +5636,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="B3:B10"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B17:B18"/>
     <mergeCell ref="B48:B52"/>
     <mergeCell ref="K53:N53"/>
     <mergeCell ref="K54:N54"/>
@@ -5691,11 +5648,6 @@
     <mergeCell ref="B36:B37"/>
     <mergeCell ref="B38:B46"/>
     <mergeCell ref="B22:B35"/>
-    <mergeCell ref="A1:U1"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="B3:B10"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="B17:B18"/>
   </mergeCells>
   <conditionalFormatting sqref="U42">
     <cfRule type="dataBar" priority="24">
@@ -5779,7 +5731,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P3:P14 P54 P16:P52">
+  <conditionalFormatting sqref="P3:P52 P54">
     <cfRule type="dataBar" priority="91">
       <dataBar>
         <cfvo type="min"/>
@@ -5876,28 +5828,28 @@
     <hyperlink ref="N7" r:id="rId26"/>
     <hyperlink ref="N13" r:id="rId27"/>
     <hyperlink ref="N16" r:id="rId28"/>
-    <hyperlink ref="N19" r:id="rId29"/>
-    <hyperlink ref="N22" r:id="rId30"/>
-    <hyperlink ref="N23" r:id="rId31"/>
-    <hyperlink ref="N26" r:id="rId32"/>
-    <hyperlink ref="N28" r:id="rId33"/>
-    <hyperlink ref="N29" r:id="rId34"/>
-    <hyperlink ref="N30" r:id="rId35"/>
-    <hyperlink ref="N31" r:id="rId36"/>
-    <hyperlink ref="N33" r:id="rId37"/>
-    <hyperlink ref="N34" r:id="rId38"/>
-    <hyperlink ref="N35" r:id="rId39"/>
-    <hyperlink ref="N37" r:id="rId40"/>
-    <hyperlink ref="N24" r:id="rId41"/>
-    <hyperlink ref="N42" r:id="rId42"/>
-    <hyperlink ref="N8" r:id="rId43"/>
-    <hyperlink ref="N10" r:id="rId44"/>
+    <hyperlink ref="N22" r:id="rId29"/>
+    <hyperlink ref="N23" r:id="rId30"/>
+    <hyperlink ref="N26" r:id="rId31"/>
+    <hyperlink ref="N28" r:id="rId32"/>
+    <hyperlink ref="N29" r:id="rId33"/>
+    <hyperlink ref="N30" r:id="rId34"/>
+    <hyperlink ref="N31" r:id="rId35"/>
+    <hyperlink ref="N33" r:id="rId36"/>
+    <hyperlink ref="N34" r:id="rId37"/>
+    <hyperlink ref="N35" r:id="rId38"/>
+    <hyperlink ref="N37" r:id="rId39"/>
+    <hyperlink ref="N24" r:id="rId40"/>
+    <hyperlink ref="N8" r:id="rId41"/>
+    <hyperlink ref="N10" r:id="rId42"/>
+    <hyperlink ref="N4" r:id="rId43"/>
+    <hyperlink ref="N32" r:id="rId44"/>
     <hyperlink ref="N15" r:id="rId45"/>
-    <hyperlink ref="N40" r:id="rId46"/>
-    <hyperlink ref="N52" r:id="rId47"/>
-    <hyperlink ref="N51" r:id="rId48"/>
-    <hyperlink ref="N4" r:id="rId49"/>
-    <hyperlink ref="N32" r:id="rId50"/>
+    <hyperlink ref="N19" r:id="rId46"/>
+    <hyperlink ref="N40" r:id="rId47"/>
+    <hyperlink ref="N42" r:id="rId48"/>
+    <hyperlink ref="N51" r:id="rId49"/>
+    <hyperlink ref="N52" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId51"/>
@@ -5980,7 +5932,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>P3:P14 P54 P16:P52</xm:sqref>
+          <xm:sqref>P3:P52 P54</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{2F6B6F4F-BC31-4B63-B3A8-F7820745DC3B}">

</xml_diff>